<commit_message>
💎 Upgrade POUPE Pro: 60+ templates com conteúdo profissional pesado gerados a partir de fontes Markdown
</commit_message>
<xml_diff>
--- a/templates/02_financeiro/01_relatorio_financeiro_mensal.xlsx
+++ b/templates/02_financeiro/01_relatorio_financeiro_mensal.xlsx
@@ -4,14 +4,73 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Relatório Mensal" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Resumo" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Receitas" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Despesas" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="49">
+  <si>
+    <t>Mês</t>
+  </si>
+  <si>
+    <t>Receitas</t>
+  </si>
+  <si>
+    <t>Despesas</t>
+  </si>
+  <si>
+    <t>Saldo</t>
+  </si>
+  <si>
+    <t>% Lucratividade</t>
+  </si>
+  <si>
+    <t>Janeiro</t>
+  </si>
+  <si>
+    <t>10000</t>
+  </si>
+  <si>
+    <t>6000</t>
+  </si>
+  <si>
+    <t>4000</t>
+  </si>
+  <si>
+    <t>40%</t>
+  </si>
+  <si>
+    <t>Fevereiro</t>
+  </si>
+  <si>
+    <t>12000</t>
+  </si>
+  <si>
+    <t>7000</t>
+  </si>
+  <si>
+    <t>5000</t>
+  </si>
+  <si>
+    <t>41.6%</t>
+  </si>
+  <si>
+    <t>Março</t>
+  </si>
+  <si>
+    <t>[PREENCHER]</t>
+  </si>
+  <si>
+    <t>[FÓRMULA: B-C]</t>
+  </si>
+  <si>
+    <t>[FÓRMULA: D/B]</t>
+  </si>
   <si>
     <t>Data</t>
   </si>
@@ -19,25 +78,88 @@
     <t>Descrição</t>
   </si>
   <si>
-    <t>Moeda</t>
+    <t>Categoria</t>
   </si>
   <si>
     <t>Valor (R$)</t>
   </si>
   <si>
-    <t>[DD/MM]</t>
-  </si>
-  <si>
-    <t>[CATEGORIA]</t>
-  </si>
-  <si>
-    <t>BRL</t>
-  </si>
-  <si>
-    <t>TOTAL:</t>
-  </si>
-  <si>
-    <t/>
+    <t>05/01/2026</t>
+  </si>
+  <si>
+    <t>Pagamento Projeto A</t>
+  </si>
+  <si>
+    <t>Serviços</t>
+  </si>
+  <si>
+    <t>15/01/2026</t>
+  </si>
+  <si>
+    <t>Venda Produto X</t>
+  </si>
+  <si>
+    <t>Vendas</t>
+  </si>
+  <si>
+    <t>2500</t>
+  </si>
+  <si>
+    <t>20/01/2026</t>
+  </si>
+  <si>
+    <t>Consultoria Y</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>02/01/2026</t>
+  </si>
+  <si>
+    <t>Aluguel Escritório</t>
+  </si>
+  <si>
+    <t>Fixo</t>
+  </si>
+  <si>
+    <t>1500</t>
+  </si>
+  <si>
+    <t>Pago</t>
+  </si>
+  <si>
+    <t>10/01/2026</t>
+  </si>
+  <si>
+    <t>Internet/Telefone</t>
+  </si>
+  <si>
+    <t>Mensal</t>
+  </si>
+  <si>
+    <t>200</t>
+  </si>
+  <si>
+    <t>Marketing (Ads)</t>
+  </si>
+  <si>
+    <t>Variável</t>
+  </si>
+  <si>
+    <t>1000</t>
+  </si>
+  <si>
+    <t>Pendente</t>
+  </si>
+  <si>
+    <t>Software SaaS</t>
+  </si>
+  <si>
+    <t>Assinatura</t>
+  </si>
+  <si>
+    <t>300</t>
   </si>
 </sst>
 </file>
@@ -55,7 +177,6 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="3">
@@ -85,9 +206,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -427,55 +546,247 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="30" customWidth="1"/>
-    <col min="3" max="3" width="8" customWidth="1"/>
-    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="1" max="5" width="20" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="4" width="20" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>24</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2">
-        <v>0</v>
+        <v>25</v>
+      </c>
+      <c r="D2" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="C3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3">
-        <f>SUM(D2:D100)</f>
+        <v>28</v>
+      </c>
+      <c r="D3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="5" width="20" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D5" t="s">
+        <v>48</v>
+      </c>
+      <c r="E5" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>